<commit_message>
Update tracker and competitive comparison for audit pack and progression
Tracker 67 to 72 completed; two rows that shipped on 09-10 and were never moved out of Pending/On Hold are now closed. Comparison: report pack Partial to Built, Student Progression Not Built to Partial - 25 Built, 7 Partial, 20 Not Built. Corrects the 'five generators' and 'no new data needed' claims, both of which were wrong.
</commit_message>
<xml_diff>
--- a/docs/FlightLogger_vs_FlightPro_Manager_Comparison_2026-09-10.xlsx
+++ b/docs/FlightLogger_vs_FlightPro_Manager_Comparison_2026-09-10.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-10, updated 2026-09-11</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>commit cf3e172 (main), 67+ completed tracker items</t>
+          <t>working tree ahead of cf3e172 (main); 72 completed tracker items</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -656,7 +656,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>3 of 4 P1 gaps closed; billing is the only P1 left</t>
+          <t>3 of 4 P1 gaps closed; billing is the only P1 left. Report pack closed 2026-09-11.</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -862,12 +862,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Regulator-ready compliance report pack</t>
+          <t>Student Progression / pace-vs-target monitoring</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Compliance &amp; Reporting</t>
+          <t>Student &amp; Training</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -877,12 +877,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Yes (EASA/FAA/CASA)</t>
+          <t>Yes (add-on, Nov 2025)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>No single bundled export. CHEAPEST REAL WIN ON THE BOARD — mostly wiring existing generators together, and one pack is what an inspector actually asks for.</t>
+          <t>PARTIAL. The projection half is built; the plan half is not, and CANNOT be without new data: training_programs has no course duration and students.joinedDate is optional and currently null on every row. Phase 2 adds both. Note this row previously claimed pace-vs-target was 'a computed view, not new data' — that was wrong.</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Student Progression / pace-vs-target monitoring</t>
+          <t>Competency-Based Training &amp; Assessment (CBTA)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -909,12 +909,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Yes (add-on, Nov 2025)</t>
+          <t>Yes (CBTA Pro)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>NEW FlightLogger feature. Genuinely useful and cheap-ish: FPM already has hours, dates and targets — this is a computed view, not new data.</t>
+          <t>Only worth building if DGCA or FTO SOP requires it. Confirm before scoping.</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Competency-Based Training &amp; Assessment (CBTA)</t>
+          <t>Learning Management System (content, quizzes)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Yes (CBTA Pro)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Only worth building if DGCA or FTO SOP requires it. Confirm before scoping.</t>
+          <t>Real gap if in-app content delivery is wanted. Needs a scoping decision first.</t>
         </is>
       </c>
     </row>
@@ -958,12 +958,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Learning Management System (content, quizzes)</t>
+          <t>Hard enforcement — block booking an overdue aircraft</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Student &amp; Training</t>
+          <t>Aircraft &amp; Maintenance</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Implied</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Real gap if in-app content delivery is wanted. Needs a scoping decision first.</t>
+          <t>Phase 2. Precondition now met (Phase 1 clean in production since 08-27). Needs two decisions: which items hard-block, and how a false-positive baseline is handled before auto-grounding.</t>
         </is>
       </c>
     </row>
@@ -990,12 +990,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Hard enforcement — block booking an overdue aircraft</t>
+          <t>Business Insights / analytics</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Aircraft &amp; Maintenance</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1005,34 +1005,34 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Implied</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Phase 2. Precondition now met (Phase 1 clean in production since 08-27). Needs two decisions: which items hard-block, and how a false-positive baseline is handled before auto-grounding.</t>
+          <t>No fleet-utilisation, instructor-productivity or revenue dashboards. Revenue half gated on Billing.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Business Insights / analytics</t>
+          <t>Online self-service booking (student-initiated)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Scheduling &amp; Operations</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Not Built</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>No fleet-utilisation, instructor-productivity or revenue dashboards. Revenue half gated on Billing.</t>
+          <t>Still unresolved: whether students can create their own bookings. A five-minute answer that may or may not create work. Backlog #14.</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Online self-service booking (student-initiated)</t>
+          <t>Room / simulator / resource booking</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Still unresolved: whether students can create their own bookings. A five-minute answer that may or may not create work. Backlog #14.</t>
+          <t>No generic classroom/room booking; could reuse the aircraft flow if needed.</t>
         </is>
       </c>
     </row>
@@ -1086,12 +1086,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Room / simulator / resource booking</t>
+          <t>Flight Time Limitation (FTL) / duty tracking</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Scheduling &amp; Operations</t>
+          <t>People / Instructors</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>No generic classroom/room booking; could reuse the aircraft flow if needed.</t>
+          <t>DELIBERATELY non-regulatory. DGCA FTL CAR was researched and found scoped to commercial air-transport crew, not FTO instructors. Reclassify only if DGCA confirms otherwise.</t>
         </is>
       </c>
     </row>
@@ -1118,12 +1118,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Flight Time Limitation (FTL) / duty tracking</t>
+          <t>Audit trail</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>People / Instructors</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>DELIBERATELY non-regulatory. DGCA FTL CAR was researched and found scoped to commercial air-transport crew, not FTO instructors. Reclassify only if DGCA confirms otherwise.</t>
+          <t>No general-purpose audit log across all tables.</t>
         </is>
       </c>
     </row>
@@ -1150,12 +1150,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Audit trail</t>
+          <t>Digital sign-offs on lessons/exams</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Compliance &amp; Reporting</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>No general-purpose audit log across all tables.</t>
+          <t>Functionally a sign-off and an audit trail; not an e-signature artifact.</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1182,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Digital sign-offs on lessons/exams</t>
+          <t>Dedicated mobile app / PWA</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Compliance &amp; Reporting</t>
+          <t>Technical / Platform</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes (mobile access)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Functionally a sign-off and an audit trail; not an e-signature artifact.</t>
+          <t>Installability (manifest, service worker, offline) not built.</t>
         </is>
       </c>
     </row>
@@ -1214,27 +1214,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Dedicated mobile app / PWA</t>
+          <t>Calendar sync (Google/Outlook)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Technical / Platform</t>
+          <t>Scheduling &amp; Operations</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Not Built</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Yes (mobile access)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Installability (manifest, service worker, offline) not built.</t>
+          <t>No external calendar sync. Integration feature, not a daily-ops gap at this scale.</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Calendar sync (Google/Outlook)</t>
+          <t>Recurring / automated scheduling</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>No external calendar sync. Integration feature, not a daily-ops gap at this scale.</t>
+          <t>No recurring-lesson templates.</t>
         </is>
       </c>
     </row>
@@ -1278,12 +1278,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Recurring / automated scheduling</t>
+          <t>Combined flight + ground syllabus in one program</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Scheduling &amp; Operations</t>
+          <t>Student &amp; Training</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes (NEW Jun 2026)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>No recurring-lesson templates.</t>
+          <t>NEW FlightLogger feature since the last analysis. Low urgency — the data exists in both modules, only a unified view is missing.</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Combined flight + ground syllabus in one program</t>
+          <t>AI-powered performance summaries</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1325,12 +1325,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Yes (NEW Jun 2026)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>NEW FlightLogger feature since the last analysis. Low urgency — the data exists in both modules, only a unified view is missing.</t>
+          <t>Progress shown as raw hours/percentages.</t>
         </is>
       </c>
     </row>
@@ -1342,12 +1342,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>AI-powered performance summaries</t>
+          <t>Employee timesheets</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Student &amp; Training</t>
+          <t>People / Instructors</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Progress shown as raw hours/percentages.</t>
+          <t>No staff timesheet/payroll-style logging.</t>
         </is>
       </c>
     </row>
@@ -1374,12 +1374,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Employee timesheets</t>
+          <t>DGCA Incident Report (statutory fields)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>People / Instructors</t>
+          <t>Compliance &amp; Reporting</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1389,12 +1389,12 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>N/A (region-specific)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>No staff timesheet/payroll-style logging.</t>
+          <t>Researched, designed and PARKED by the user 2026-09-10. Legal basis established: G.S.R. 829(E), Rule 4(2), eleven notification items. Unblocked whenever it is picked up.</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>DGCA Incident Report (statutory fields)</t>
+          <t>Customizable / user-built report templates</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1421,12 +1421,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>N/A (region-specific)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Researched, designed and PARKED by the user 2026-09-10. Legal basis established: G.S.R. 829(E), Rule 4(2), eleven notification items. Unblocked whenever it is picked up.</t>
+          <t>Adding a report type needs a code change.</t>
         </is>
       </c>
     </row>
@@ -1438,12 +1438,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Customizable / user-built report templates</t>
+          <t>Accounting integration (QuickBooks)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Compliance &amp; Reporting</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Adding a report type needs a code change.</t>
+          <t>Defer well past a basic ledger.</t>
         </is>
       </c>
     </row>
@@ -1470,12 +1470,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Accounting integration (QuickBooks)</t>
+          <t>Internal messaging / announcements</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Communication</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Defer well past a basic ledger.</t>
+          <t>No in-app messaging.</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Internal messaging / announcements</t>
+          <t>Document / content library</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>No in-app messaging.</t>
+          <t>A simple Documents tab under Admin Setup would cover most of the need.</t>
         </is>
       </c>
     </row>
@@ -1534,12 +1534,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Document / content library</t>
+          <t>Public API for integrations</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Communication</t>
+          <t>Technical / Platform</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>A simple Documents tab under Admin Setup would cover most of the need.</t>
+          <t>No documented public API.</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Public API for integrations</t>
+          <t>Single sign-on (SSO)</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>No documented public API.</t>
+          <t>No SAML/OAuth org login.</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Single sign-on (SSO)</t>
+          <t>Multi-location / multi-campus</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>No SAML/OAuth org login.</t>
+          <t>Touches most of the data model. Not needed unless the FTO opens a second base.</t>
         </is>
       </c>
     </row>
@@ -1630,12 +1630,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Multi-location / multi-campus</t>
+          <t>Checkbox-style Requirements UI</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Technical / Platform</t>
+          <t>Student &amp; Training</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -1645,12 +1645,12 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Touches most of the data model. Not needed unless the FTO opens a second base.</t>
+          <t>Backlog #1. Friendlier requirement completion than today's checklist. Smallest self-contained backlog item.</t>
         </is>
       </c>
     </row>
@@ -1662,12 +1662,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Checkbox-style Requirements UI</t>
+          <t>Multi-language support (i18n)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Student &amp; Training</t>
+          <t>Technical / Platform</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Backlog #1. Friendlier requirement completion than today's checklist. Smallest self-contained backlog item.</t>
+          <t>Backlog #7. No framework, no translated strings. No demand signal yet — lowest priority.</t>
         </is>
       </c>
     </row>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Multi-language support (i18n)</t>
+          <t>One-time 'unrecognized Model' admin banner</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Technical / Platform</t>
+          <t>Aircraft &amp; Maintenance</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Backlog #7. No framework, no translated strings. No demand signal yet — lowest priority.</t>
+          <t>Backlog #9. Only covers EXISTING aircraft predating the warn-and-block fix; new ones can no longer be saved with a bad Model.</t>
         </is>
       </c>
     </row>
@@ -1726,12 +1726,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>One-time 'unrecognized Model' admin banner</t>
+          <t>GET /api/maintenance-records route</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Aircraft &amp; Maintenance</t>
+          <t>Technical / Platform</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Backlog #9. Only covers EXISTING aircraft predating the warn-and-block fix; new ones can no longer be saved with a bad Model.</t>
+          <t>Maintenance READS still go through a legacy direct client-side Supabase call; only writes are routed through the API.</t>
         </is>
       </c>
     </row>
@@ -1758,12 +1758,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>GET /api/maintenance-records route</t>
+          <t>Log Book Serial No. / CAMO Approval No. — real values</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Technical / Platform</t>
+          <t>Compliance &amp; Reporting</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Maintenance READS still go through a legacy direct client-side Supabase call; only writes are routed through the API.</t>
+          <t>Placeholder fields shipped 2026-09-10. BLOCKED on the user's real log book cover and CAMO/AMO approval certificate.</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Log Book Serial No. / CAMO Approval No. — real values</t>
+          <t>Other reports still export CSV labelled 'Excel'</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -1809,38 +1809,6 @@
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>Placeholder fields shipped 2026-09-10. BLOCKED on the user's real log book cover and CAMO/AMO approval certificate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Other reports still export CSV labelled 'Excel'</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Compliance &amp; Reporting</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Not Built</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>Daily Flying and BA reports emit CSV while saying Excel/CSV. Maintenance Log already exports real styled .xlsx.</t>
         </is>
@@ -1858,7 +1826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1907,7 +1875,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>✅ CODE FIXED 2026-09-10 — ConfirmDialog Escape + 5 missing aria-labels. Accessible names verified in the a11y tree; NO SCREEN READER WAS RUN. Reword the row rather than re-ticking it.</t>
+          <t>CODE FIXED 2026-09-10 (4964989) — ConfirmDialog Escape + a shared listener stack + 5 missing aria-labels. PARTIALLY VERIFIED 2026-09-11: Escape confirmed closing the Maintenance edit modal in a real browser. STILL OPEN: the other 14 modals, and no screen reader has been run at all — accessible names were checked in the accessibility tree only. Do not mark this verified on tree inspection alone.</t>
         </is>
       </c>
     </row>
@@ -2315,37 +2283,15 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Compliance</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Item 66 — quick-reschedule buttons</t>
+          <t>NOTAM disclaimer in the printed briefing</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Maintenance page '+4h'/'+1d' don't visibly move a SCHEDULED record. Not root-caused; the Edit modal works.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Compliance</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>NOTAM disclaimer in the printed briefing</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Restored 2026-09-10 and verified in source only — that markup renders only when NOTAMs are active.</t>
         </is>
@@ -2776,17 +2722,17 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Not Built</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Progress page shows cumulative hours and % against requirements. No comparison of actual pace vs required pace, no cohort view.</t>
+          <t>Progress page shows a PROJECTED FINISH from the rate actually flown over a trailing 8 weeks, with sample size, a stalled flag, and a 2-year cap. Shipped 2026-09-11.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>NEW FlightLogger feature. Genuinely useful and cheap-ish: FPM already has hours, dates and targets — this is a computed view, not new data.</t>
+          <t>PARTIAL. The projection half is built; the plan half is not, and CANNOT be without new data: training_programs has no course duration and students.joinedDate is optional and currently null on every row. Phase 2 adds both. Note this row previously claimed pace-vs-target was 'a computed view, not new data' — that was wrong.</t>
         </is>
       </c>
     </row>
@@ -3576,17 +3522,17 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Five working generators: Daily Flying, BA Register, BA Report, Student Logbook, Maintenance Log (PDF + XLSX).</t>
+          <t>DGCA Audit Pack (/dashboard/reports/audit-pack), shipped 2026-09-11: one PDF for a date range bundling every saved Daily Flying Report, the BA register rollup, and the Maintenance Log for each aircraft with completed work. FOUR generators, not five as this row previously said — the BA Register page exports CSV only and has no PDF generator; the pack uses the BA Report rollup, which covers the same data over a range.</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>No single bundled export. CHEAPEST REAL WIN ON THE BOARD — mostly wiring existing generators together, and one pack is what an inspector actually asks for.</t>
+          <t>CLOSED 2026-09-11. Days with no saved Daily Flying Report are listed on the cover rather than omitted, so a pack with holes says so. Student logbooks deliberately excluded (per-student; a month across 20 students runs to hundreds of pages) — still exported individually. Range capped at 92 days.</t>
         </is>
       </c>
     </row>
@@ -4202,22 +4148,22 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>No consolidated DGCA audit-pack export</t>
+          <t>No consolidated DGCA audit-pack export — CLOSED 2026-09-11</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>An inspection wants one pack, not five separate pages. Five generators already work.</t>
+          <t>An inspection wants one pack, not five separate pages. SHIPPED 2026-09-11 as the DGCA Audit Pack (/dashboard/reports/audit-pack) and verified live.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Single 'Compliance Export' page bundling the existing PDF/XLSX generators for a date range. Mostly wiring.</t>
+          <t>Done. Note for anyone reading the old wording: there are FOUR PDF generators, not five — the BA Register page has CSV export only. The pack uses the BA Report rollup instead.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Small — CHEAPEST WIN</t>
+          <t>Small — DONE</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4914,6 +4860,72 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Regulator-ready compliance report pack</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 — DGCA Audit Pack. Was flagged here as the cheapest real win; it was.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Quick-reschedule stale OVERDUE state</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Open bug</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Fixed + verified</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 — SWR cache splice was not revalidating derived fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Student Progression / pace-vs-target</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Not Built</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11 — projection half shipped; plan half needs course duration + joined dates</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Escape to a 16th uncounted modal; test the stack; empty-day placeholder on Daily Flying PDF
MaintenanceDueSection's Set Baseline / Log Completion modal had click-outside and a labelled Close button but no Escape handling, and was never in the documented count of 15. All 16 overlays now call useEscapeToClose. Adds a unit test for the stack behaviour, which fixed a real bug on 09-10 but is unreachable in the UI and was exercised by nothing. Daily Flying PDF now prints a placeholder row for a day with no flights instead of a bare header bar.
</commit_message>
<xml_diff>
--- a/docs/FlightLogger_vs_FlightPro_Manager_Comparison_2026-09-10.xlsx
+++ b/docs/FlightLogger_vs_FlightPro_Manager_Comparison_2026-09-10.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>working tree ahead of cf3e172 (main); 72 completed tracker items</t>
+          <t>working tree ahead of 609b625 (main); 73 completed tracker items</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1870,12 +1870,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Screen-reader verification of modals and Close buttons</t>
+          <t>Screen-reader pass (13/16 Escape now verified)</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>CODE FIXED 2026-09-10 (4964989) — ConfirmDialog Escape + a shared listener stack + 5 missing aria-labels. PARTIALLY VERIFIED 2026-09-11: Escape confirmed closing the Maintenance edit modal in a real browser. STILL OPEN: the other 14 modals, and no screen reader has been run at all — accessible names were checked in the accessibility tree only. Do not mark this verified on tree inspection alone.</t>
+          <t>VERIFIED 2026-09-11 by driving the running app: 13 of 16 overlay modals confirmed closing on a REAL Escape keypress (Aircraft, Student, Instructor, FuelLog, Availability, FlightRecord, Booking, UserEdit, UserPermissions, GroundSchool 'New Ground Class', ConfirmDialog, MaintenanceForm, FlightDetail). ConfirmDialog also confirmed cancelling without deleting (32 rows intact). THE COUNT WAS 15 AND IS ACTUALLY 16 — MaintenanceDueSection's Set Baseline / Log Completion modal was never counted and had NO Escape handling; fixed 2026-09-11 (useEscapeToClose's own header had warned the pattern would drift 'the next time a 16th modal is added', and it did). STILL UNVERIFIED: (1) that new modal — MaintenanceDueSection renders null while every item is OK, the same blocker as item 76; (2) DebriefForm — its button is time-gated, 'Opens 19:00 IST', and the booking form refuses an already-ended flight; (3) the RequirementsChecklist modal — the Progress page renders that checklist read-only. ALSO STILL UNVERIFIED: the stacked case (a ConfirmDialog over another modal), which the hook's stack exists for — it is NOT REACHABLE in the current UI; the only two ConfirmDialog call sites sit over a page, and FlightDetailModal's cancel-reason picker renders inside the same overlay. No unit test covers it either. AND NO SCREEN READER HAS BEEN RUN — that half is untouched.</t>
         </is>
       </c>
     </row>
@@ -2294,6 +2294,28 @@
       <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Restored 2026-09-10 and verified in source only — that markup renders only when NOTAMs are active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>NOTAM disclaimer in the printed briefing — CLEARED 2026-09-11</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Verified live: with 79 active NOTAMs showing, the on-screen panel rendered both the disclaimer and the '+79 more — see the full briefing' truncation notice. The PRINT path carries its own disclaimer with different wording ('Situational awareness only — this is not an official pre-flight briefing. Verify against AIM India') and its own truncation disclosure in the heading ('N total, first 3 shown') — confirmed in source; not rendered, because Print Brief opens a window and a print dialog.</t>
         </is>
       </c>
     </row>

</xml_diff>